<commit_message>
loader added to login page
</commit_message>
<xml_diff>
--- a/storage/app/Colombo_re_upload.xlsx
+++ b/storage/app/Colombo_re_upload.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="53">
   <si>
     <t>#</t>
   </si>
@@ -95,16 +95,22 @@
     <t>3/21/2025</t>
   </si>
   <si>
-    <t>A</t>
+    <t>P3</t>
   </si>
   <si>
-    <t>B</t>
+    <t>Executive</t>
   </si>
   <si>
-    <t>t</t>
+    <t>LK</t>
   </si>
   <si>
-    <t>cf</t>
+    <t>0112256789</t>
+  </si>
+  <si>
+    <t>Gayan</t>
+  </si>
+  <si>
+    <t>Nimali</t>
   </si>
   <si>
     <t>s</t>
@@ -119,10 +125,55 @@
     <t>RE2</t>
   </si>
   <si>
+    <t>P4</t>
+  </si>
+  <si>
+    <t>Support Team</t>
+  </si>
+  <si>
+    <t>0112256787</t>
+  </si>
+  <si>
     <t>RE3</t>
   </si>
   <si>
+    <t>P5</t>
+  </si>
+  <si>
+    <t>Intern</t>
+  </si>
+  <si>
     <t>RE4</t>
+  </si>
+  <si>
+    <t>P6</t>
+  </si>
+  <si>
+    <t>Senior</t>
+  </si>
+  <si>
+    <t>RE5</t>
+  </si>
+  <si>
+    <t>P7</t>
+  </si>
+  <si>
+    <t>Junior</t>
+  </si>
+  <si>
+    <t>RE6</t>
+  </si>
+  <si>
+    <t>P8</t>
+  </si>
+  <si>
+    <t>Senior Engineer</t>
+  </si>
+  <si>
+    <t>RE7</t>
+  </si>
+  <si>
+    <t>P9</t>
   </si>
 </sst>
 </file>
@@ -539,35 +590,35 @@
       <c r="B2" t="s">
         <v>25</v>
       </c>
-      <c r="C2">
-        <v>3</v>
+      <c r="C2" t="s">
+        <v>26</v>
       </c>
-      <c r="D2">
-        <v>4</v>
+      <c r="D2" t="s">
+        <v>27</v>
       </c>
       <c r="E2">
         <v>6</v>
       </c>
       <c r="F2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="G2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="H2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="I2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="J2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="K2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="L2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="M2"/>
       <c r="N2"/>
@@ -584,22 +635,32 @@
     </row>
     <row r="3" spans="1:24">
       <c r="A3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B3" t="s">
         <v>25</v>
       </c>
-      <c r="C3">
-        <v>4</v>
+      <c r="C3" t="s">
+        <v>36</v>
       </c>
-      <c r="D3">
-        <v>5</v>
+      <c r="D3" t="s">
+        <v>37</v>
       </c>
-      <c r="E3"/>
-      <c r="F3"/>
-      <c r="G3"/>
-      <c r="H3"/>
-      <c r="I3"/>
+      <c r="E3">
+        <v>7</v>
+      </c>
+      <c r="F3" t="s">
+        <v>28</v>
+      </c>
+      <c r="G3" t="s">
+        <v>38</v>
+      </c>
+      <c r="H3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I3" t="s">
+        <v>31</v>
+      </c>
       <c r="J3"/>
       <c r="K3"/>
       <c r="L3"/>
@@ -618,22 +679,32 @@
     </row>
     <row r="4" spans="1:24">
       <c r="A4" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="B4" t="s">
         <v>25</v>
       </c>
-      <c r="C4">
-        <v>5</v>
+      <c r="C4" t="s">
+        <v>40</v>
       </c>
-      <c r="D4">
-        <v>6</v>
+      <c r="D4" t="s">
+        <v>41</v>
       </c>
-      <c r="E4"/>
-      <c r="F4"/>
-      <c r="G4"/>
-      <c r="H4"/>
-      <c r="I4"/>
+      <c r="E4">
+        <v>8</v>
+      </c>
+      <c r="F4" t="s">
+        <v>28</v>
+      </c>
+      <c r="G4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I4" t="s">
+        <v>31</v>
+      </c>
       <c r="J4"/>
       <c r="K4"/>
       <c r="L4"/>
@@ -652,22 +723,32 @@
     </row>
     <row r="5" spans="1:24">
       <c r="A5" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="B5" t="s">
         <v>25</v>
       </c>
-      <c r="C5">
-        <v>6</v>
+      <c r="C5" t="s">
+        <v>43</v>
       </c>
-      <c r="D5">
-        <v>7</v>
+      <c r="D5" t="s">
+        <v>44</v>
       </c>
-      <c r="E5"/>
-      <c r="F5"/>
-      <c r="G5"/>
-      <c r="H5"/>
-      <c r="I5"/>
+      <c r="E5">
+        <v>9</v>
+      </c>
+      <c r="F5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H5" t="s">
+        <v>30</v>
+      </c>
+      <c r="I5" t="s">
+        <v>31</v>
+      </c>
       <c r="J5"/>
       <c r="K5"/>
       <c r="L5"/>
@@ -685,21 +766,33 @@
       <c r="X5"/>
     </row>
     <row r="6" spans="1:24">
-      <c r="A6"/>
+      <c r="A6" t="s">
+        <v>45</v>
+      </c>
       <c r="B6" t="s">
         <v>25</v>
       </c>
-      <c r="C6">
-        <v>7</v>
+      <c r="C6" t="s">
+        <v>46</v>
       </c>
-      <c r="D6">
-        <v>8</v>
+      <c r="D6" t="s">
+        <v>47</v>
       </c>
-      <c r="E6"/>
-      <c r="F6"/>
-      <c r="G6"/>
-      <c r="H6"/>
-      <c r="I6"/>
+      <c r="E6">
+        <v>10</v>
+      </c>
+      <c r="F6" t="s">
+        <v>28</v>
+      </c>
+      <c r="G6" t="s">
+        <v>29</v>
+      </c>
+      <c r="H6" t="s">
+        <v>30</v>
+      </c>
+      <c r="I6" t="s">
+        <v>31</v>
+      </c>
       <c r="J6"/>
       <c r="K6"/>
       <c r="L6"/>
@@ -717,21 +810,33 @@
       <c r="X6"/>
     </row>
     <row r="7" spans="1:24">
-      <c r="A7"/>
+      <c r="A7" t="s">
+        <v>48</v>
+      </c>
       <c r="B7" t="s">
         <v>25</v>
       </c>
-      <c r="C7">
-        <v>8</v>
+      <c r="C7" t="s">
+        <v>49</v>
       </c>
-      <c r="D7">
-        <v>9</v>
+      <c r="D7" t="s">
+        <v>50</v>
       </c>
-      <c r="E7"/>
-      <c r="F7"/>
-      <c r="G7"/>
-      <c r="H7"/>
-      <c r="I7"/>
+      <c r="E7">
+        <v>11</v>
+      </c>
+      <c r="F7" t="s">
+        <v>28</v>
+      </c>
+      <c r="G7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H7" t="s">
+        <v>30</v>
+      </c>
+      <c r="I7" t="s">
+        <v>31</v>
+      </c>
       <c r="J7"/>
       <c r="K7"/>
       <c r="L7"/>
@@ -749,19 +854,33 @@
       <c r="X7"/>
     </row>
     <row r="8" spans="1:24">
-      <c r="A8"/>
+      <c r="A8" t="s">
+        <v>51</v>
+      </c>
       <c r="B8" t="s">
         <v>25</v>
       </c>
-      <c r="C8">
-        <v>9</v>
+      <c r="C8" t="s">
+        <v>52</v>
       </c>
-      <c r="D8"/>
-      <c r="E8"/>
-      <c r="F8"/>
-      <c r="G8"/>
-      <c r="H8"/>
-      <c r="I8"/>
+      <c r="D8" t="s">
+        <v>50</v>
+      </c>
+      <c r="E8">
+        <v>12</v>
+      </c>
+      <c r="F8" t="s">
+        <v>28</v>
+      </c>
+      <c r="G8" t="s">
+        <v>29</v>
+      </c>
+      <c r="H8" t="s">
+        <v>30</v>
+      </c>
+      <c r="I8" t="s">
+        <v>31</v>
+      </c>
       <c r="J8"/>
       <c r="K8"/>
       <c r="L8"/>

</xml_diff>